<commit_message>
fix(site): rework template, form, and print pages
Show blank templates as column lists with the guide's notes. Let tables
use the page width and size columns to their text. Add tick boxes and
text fields to the checklists, a fillable statement of applicability,
print icons, and Download my answers so typed answers can be kept.

Fixes #13

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjzbFX8BVBbwU7jJMPUWj5
</commit_message>
<xml_diff>
--- a/site/docs/sam-toolkit/audit-and-review-checklist.xlsx
+++ b/site/docs/sam-toolkit/audit-and-review-checklist.xlsx
@@ -181,6 +181,11 @@
       </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C2:C5">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+  </dataValidations>
 </worksheet>
 </file>
 
@@ -539,6 +544,11 @@
       </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C2:C4">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+  </dataValidations>
 </worksheet>
 </file>
 
@@ -750,6 +760,11 @@
       </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C2:C9">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+  </dataValidations>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
fix(site): rework template, form, and print pages (#14)
Fixes the document pages you flagged: renewal calendar, authorization
log, vendor register, asset record, license position, statement of
applicability, and the audit checklist.

- Blank CSV templates show their columns as a list, with the guide's
notes.
- Tables use the page width and size columns to their text.
- Checklists get tick boxes (Done, Prepared) and text fields (Notes,
Evidence).
- The statement of applicability is a fillable form with an in-scope
count and a CSV download of the answers.
- Print icons at the top and bottom right of every document page.
- Download my answers (Word) keeps typed answers; a note on each page
says the Word and Excel downloads are blank copies.

make test, make build, and make scan pass.

Fixes #13

🤖 Generated with [Claude Code](https://claude.com/claude-code)

https://claude.ai/code/session_01XjzbFX8BVBbwU7jJMPUWj5

---------

Co-authored-by: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/site/docs/sam-toolkit/audit-and-review-checklist.xlsx
+++ b/site/docs/sam-toolkit/audit-and-review-checklist.xlsx
@@ -181,6 +181,11 @@
       </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C2:C5">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+  </dataValidations>
 </worksheet>
 </file>
 
@@ -539,6 +544,11 @@
       </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C2:C4">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+  </dataValidations>
 </worksheet>
 </file>
 
@@ -750,6 +760,11 @@
       </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C2:C9">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+  </dataValidations>
 </worksheet>
 </file>
 

</xml_diff>